<commit_message>
Improve docs and workbook sync API
</commit_message>
<xml_diff>
--- a/marketing/sales-tracker.xlsx
+++ b/marketing/sales-tracker.xlsx
@@ -1046,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1149,6 +1149,270 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>OR-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Diego Granados</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Product Manager</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>AI / PM</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Public LinkedIn</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diegogranadosh/</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Ara</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Send AI Product Strategy syllabus + eval module teaser</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Wiley author on AI PM. Posts about AI evals. Strong fit for AI Product Strategy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>OR-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Lianna Patch</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Founder / Conversion Copywriter</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Punchline Copy</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Public LinkedIn</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/liannapatch</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Ara</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Send Launch Copy Studio offer-shape preview</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Spoke at MicroConf US on emotion in copy. Possible partner, not just student.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>OR-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Justin Welsh</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Solopreneur / Newsletter Operator</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The Saturday Solopreneur</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Public LinkedIn</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/justinwelsh/</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Ara</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Pitch cross-promo for Creator Business Kit</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>175k+ newsletter subs. Best fit as affiliate / cross-promo, not direct student.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>OR-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Alex Freberg</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Founder / Educator</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AnalystBuilder.com</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Public LinkedIn</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alex-freberg/</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Ara</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Pitch Analytics That Sell as complementary cohort</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Runs popular YouTube on data analysis. Audience overlap with Analytics That Sell.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>